<commit_message>
prueba 8 nueva organizacion
</commit_message>
<xml_diff>
--- a/pruebas/ventas.xlsx
+++ b/pruebas/ventas.xlsx
@@ -471,57 +471,57 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Aceite mineral premium para motores a gasolina</t>
+          <t>Llanta radial de alto rendimiento, bajo ruido</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>45973</v>
+        <v>45996</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G2" t="n">
-        <v>74000</v>
+        <v>250800</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Filtro de aire de alto rendimiento para SUV</t>
+          <t>Llanta radial de alto rendimiento, bajo ruido</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45973</v>
+        <v>45996</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
-        <v>120000</v>
+        <v>3009600</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B4" t="n">
         <v>1</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>45973</v>
+        <v>45996</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
         <v>285000</v>
@@ -546,7 +546,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
@@ -556,317 +556,227 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Batería de libre mantenimiento para vehículos de alto consumo</t>
+          <t>Llanta radial de alto rendimiento, bajo ruido</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>45973</v>
+        <v>45996</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>380000</v>
+        <v>256500</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Batería de libre mantenimiento para vehículos de alto consumo</t>
-        </is>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" s="2" t="n">
-        <v>45973</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
+        <v>45982</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>380000</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>13</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Batería de libre mantenimiento para vehículos de alto consumo</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" s="2" t="n">
-        <v>45973</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
+        <v>45982</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>4940000</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B8" t="n">
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Batería de libre mantenimiento para vehículos de alto consumo</t>
+          <t>Aceite mineral premium para motores a gasolina</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>1520000</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Batería de libre mantenimiento para vehículos de alto consumo</t>
+          <t>Aceite mineral premium para motores a gasolina</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>380000</v>
+        <v>148000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
+          <t>Batería de libre mantenimiento para vehículos de alto consumo</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>285000</v>
+        <v>17100000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>16</v>
-      </c>
-      <c r="B11" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
+        <v>45981</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>285000</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>17</v>
-      </c>
-      <c r="B12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
+        <v>45981</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>285000</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>18</v>
-      </c>
-      <c r="B13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Aceite mineral premium para motores a gasolina</t>
-        </is>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
+        <v>45980</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>37000</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>19</v>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>12</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
+        <v>45979</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>3420000</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>20</v>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
+        <v>45978</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>285000</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>21</v>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
+        <v>45977</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>285000</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>10</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Llanta radial de alto rendimiento, bajo ruido</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="F17" t="n">
-        <v>1</v>
-      </c>
+        <v>45976</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>2850000</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18">

</xml_diff>